<commit_message>
Primera versión — análisis sensibilidad corneal DM2
</commit_message>
<xml_diff>
--- a/resultados/base_sensibilidad_corneal_113_limpia.xlsx
+++ b/resultados/base_sensibilidad_corneal_113_limpia.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE114"/>
+  <dimension ref="A1:AF114"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="20.7109375" style="2" customWidth="1"/>
@@ -514,6 +514,11 @@
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
+          <t>control_glucemico_hba1c</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
           <t>glucemia_categoria</t>
         </is>
       </c>
@@ -647,6 +652,11 @@
       </c>
       <c r="AE2" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -780,6 +790,11 @@
       </c>
       <c r="AE3" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -913,6 +928,11 @@
       </c>
       <c r="AE4" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -1046,6 +1066,11 @@
       </c>
       <c r="AE5" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -1179,6 +1204,11 @@
       </c>
       <c r="AE6" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -1312,6 +1342,11 @@
       </c>
       <c r="AE7" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -1445,6 +1480,11 @@
       </c>
       <c r="AE8" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -1578,6 +1618,11 @@
       </c>
       <c r="AE9" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -1711,6 +1756,11 @@
       </c>
       <c r="AE10" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -1844,6 +1894,11 @@
       </c>
       <c r="AE11" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -1977,6 +2032,11 @@
       </c>
       <c r="AE12" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -2110,6 +2170,11 @@
       </c>
       <c r="AE13" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -2243,6 +2308,11 @@
       </c>
       <c r="AE14" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -2376,6 +2446,11 @@
       </c>
       <c r="AE15" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -2509,6 +2584,11 @@
       </c>
       <c r="AE16" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -2642,6 +2722,11 @@
       </c>
       <c r="AE17" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -2775,6 +2860,11 @@
       </c>
       <c r="AE18" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -2908,6 +2998,11 @@
       </c>
       <c r="AE19" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -3041,6 +3136,11 @@
       </c>
       <c r="AE20" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -3174,6 +3274,11 @@
       </c>
       <c r="AE21" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -3307,6 +3412,11 @@
       </c>
       <c r="AE22" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -3440,6 +3550,11 @@
       </c>
       <c r="AE23" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -3573,6 +3688,11 @@
       </c>
       <c r="AE24" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -3706,6 +3826,11 @@
       </c>
       <c r="AE25" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -3839,6 +3964,11 @@
       </c>
       <c r="AE26" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -3972,6 +4102,11 @@
       </c>
       <c r="AE27" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF27" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -4105,6 +4240,11 @@
       </c>
       <c r="AE28" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF28" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -4238,6 +4378,11 @@
       </c>
       <c r="AE29" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF29" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -4371,6 +4516,11 @@
       </c>
       <c r="AE30" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF30" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -4504,6 +4654,11 @@
       </c>
       <c r="AE31" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -4637,6 +4792,11 @@
       </c>
       <c r="AE32" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF32" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -4770,6 +4930,11 @@
       </c>
       <c r="AE33" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF33" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -4903,6 +5068,11 @@
       </c>
       <c r="AE34" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF34" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -5036,6 +5206,11 @@
       </c>
       <c r="AE35" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF35" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -5169,6 +5344,11 @@
       </c>
       <c r="AE36" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF36" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -5302,6 +5482,11 @@
       </c>
       <c r="AE37" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF37" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -5435,6 +5620,11 @@
       </c>
       <c r="AE38" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF38" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -5568,6 +5758,11 @@
       </c>
       <c r="AE39" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF39" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -5701,6 +5896,11 @@
       </c>
       <c r="AE40" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF40" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -5834,6 +6034,11 @@
       </c>
       <c r="AE41" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF41" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -5967,6 +6172,11 @@
       </c>
       <c r="AE42" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF42" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -6100,6 +6310,11 @@
       </c>
       <c r="AE43" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF43" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -6233,6 +6448,11 @@
       </c>
       <c r="AE44" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF44" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -6366,6 +6586,11 @@
       </c>
       <c r="AE45" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF45" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -6499,6 +6724,11 @@
       </c>
       <c r="AE46" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF46" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -6632,6 +6862,11 @@
       </c>
       <c r="AE47" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF47" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -6765,6 +7000,11 @@
       </c>
       <c r="AE48" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF48" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -6898,6 +7138,11 @@
       </c>
       <c r="AE49" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF49" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -7031,6 +7276,11 @@
       </c>
       <c r="AE50" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF50" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -7164,6 +7414,11 @@
       </c>
       <c r="AE51" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF51" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -7297,6 +7552,11 @@
       </c>
       <c r="AE52" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF52" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -7430,6 +7690,11 @@
       </c>
       <c r="AE53" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF53" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -7563,6 +7828,11 @@
       </c>
       <c r="AE54" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF54" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -7696,6 +7966,11 @@
       </c>
       <c r="AE55" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF55" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -7829,6 +8104,11 @@
       </c>
       <c r="AE56" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF56" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -7962,6 +8242,11 @@
       </c>
       <c r="AE57" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF57" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -8095,6 +8380,11 @@
       </c>
       <c r="AE58" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF58" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -8228,6 +8518,11 @@
       </c>
       <c r="AE59" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF59" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -8361,6 +8656,11 @@
       </c>
       <c r="AE60" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF60" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -8494,6 +8794,11 @@
       </c>
       <c r="AE61" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF61" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -8627,6 +8932,11 @@
       </c>
       <c r="AE62" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF62" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -8760,6 +9070,11 @@
       </c>
       <c r="AE63" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF63" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -8893,6 +9208,11 @@
       </c>
       <c r="AE64" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF64" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -9026,6 +9346,11 @@
       </c>
       <c r="AE65" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF65" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -9159,6 +9484,11 @@
       </c>
       <c r="AE66" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF66" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -9292,6 +9622,11 @@
       </c>
       <c r="AE67" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF67" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -9425,6 +9760,11 @@
       </c>
       <c r="AE68" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF68" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -9558,6 +9898,11 @@
       </c>
       <c r="AE69" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF69" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -9691,6 +10036,11 @@
       </c>
       <c r="AE70" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF70" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -9824,6 +10174,11 @@
       </c>
       <c r="AE71" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF71" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -9957,6 +10312,11 @@
       </c>
       <c r="AE72" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF72" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -10090,6 +10450,11 @@
       </c>
       <c r="AE73" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF73" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -10223,6 +10588,11 @@
       </c>
       <c r="AE74" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF74" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -10356,6 +10726,11 @@
       </c>
       <c r="AE75" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF75" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -10489,6 +10864,11 @@
       </c>
       <c r="AE76" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF76" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -10622,6 +11002,11 @@
       </c>
       <c r="AE77" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF77" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -10755,6 +11140,11 @@
       </c>
       <c r="AE78" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF78" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -10888,6 +11278,11 @@
       </c>
       <c r="AE79" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF79" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -11021,6 +11416,11 @@
       </c>
       <c r="AE80" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF80" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -11154,6 +11554,11 @@
       </c>
       <c r="AE81" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF81" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -11287,6 +11692,11 @@
       </c>
       <c r="AE82" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF82" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -11420,6 +11830,11 @@
       </c>
       <c r="AE83" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF83" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -11553,6 +11968,11 @@
       </c>
       <c r="AE84" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF84" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -11686,6 +12106,11 @@
       </c>
       <c r="AE85" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF85" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -11819,6 +12244,11 @@
       </c>
       <c r="AE86" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF86" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -11952,6 +12382,11 @@
       </c>
       <c r="AE87" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF87" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -12085,6 +12520,11 @@
       </c>
       <c r="AE88" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF88" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -12218,6 +12658,11 @@
       </c>
       <c r="AE89" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF89" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -12351,6 +12796,11 @@
       </c>
       <c r="AE90" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF90" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -12484,6 +12934,11 @@
       </c>
       <c r="AE91" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF91" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -12617,6 +13072,11 @@
       </c>
       <c r="AE92" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF92" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -12750,6 +13210,11 @@
       </c>
       <c r="AE93" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF93" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -12883,6 +13348,11 @@
       </c>
       <c r="AE94" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF94" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -13016,6 +13486,11 @@
       </c>
       <c r="AE95" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF95" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -13149,6 +13624,11 @@
       </c>
       <c r="AE96" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF96" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -13282,6 +13762,11 @@
       </c>
       <c r="AE97" t="inlineStr">
         <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF97" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -13415,6 +13900,11 @@
       </c>
       <c r="AE98" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF98" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -13548,6 +14038,11 @@
       </c>
       <c r="AE99" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF99" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -13681,6 +14176,11 @@
       </c>
       <c r="AE100" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF100" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -13814,6 +14314,11 @@
       </c>
       <c r="AE101" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF101" t="inlineStr">
+        <is>
           <t>Menor de 126 mg/dL</t>
         </is>
       </c>
@@ -13947,6 +14452,11 @@
       </c>
       <c r="AE102" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF102" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -14080,6 +14590,11 @@
       </c>
       <c r="AE103" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF103" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -14213,6 +14728,11 @@
       </c>
       <c r="AE104" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF104" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -14346,6 +14866,11 @@
       </c>
       <c r="AE105" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF105" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -14479,6 +15004,11 @@
       </c>
       <c r="AE106" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF106" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -14612,6 +15142,11 @@
       </c>
       <c r="AE107" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF107" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -14745,6 +15280,11 @@
       </c>
       <c r="AE108" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF108" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -14878,6 +15418,11 @@
       </c>
       <c r="AE109" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF109" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -15011,6 +15556,11 @@
       </c>
       <c r="AE110" t="inlineStr">
         <is>
+          <t>Muy mal controlado</t>
+        </is>
+      </c>
+      <c r="AF110" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -15144,6 +15694,11 @@
       </c>
       <c r="AE111" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF111" t="inlineStr">
+        <is>
           <t>≥200 mg/dL</t>
         </is>
       </c>
@@ -15277,6 +15832,11 @@
       </c>
       <c r="AE112" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF112" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -15410,6 +15970,11 @@
       </c>
       <c r="AE113" t="inlineStr">
         <is>
+          <t>Mal controlado</t>
+        </is>
+      </c>
+      <c r="AF113" t="inlineStr">
+        <is>
           <t>126-199 mg/dL</t>
         </is>
       </c>
@@ -15542,6 +16107,11 @@
         </is>
       </c>
       <c r="AE114" t="inlineStr">
+        <is>
+          <t>Controlado</t>
+        </is>
+      </c>
+      <c r="AF114" t="inlineStr">
         <is>
           <t>Menor de 126 mg/dL</t>
         </is>

</xml_diff>